<commit_message>
Sprint 5 Day 35: full pipeline verified end-to-end on Windows/pandas 3.0.5 - 95/95 tests passing
</commit_message>
<xml_diff>
--- a/output/valuation_summary.xlsx
+++ b/output/valuation_summary.xlsx
@@ -434,22 +434,22 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>pe_ratio</t>
+          <t>P/E</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>pb_ratio</t>
+          <t>P/B</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>ev_ebitda</t>
+          <t>EV/EBITDA</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>fcf_yield_pct</t>
+          <t>FCF_yield_pct</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -494,13 +494,13 @@
         <v>12.63</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05188004157485571</v>
+        <v>0.07127809977975783</v>
       </c>
       <c r="H2" t="n">
-        <v>62.63</v>
+        <v>60.485</v>
       </c>
       <c r="I2" t="n">
-        <v>58.38222967309304</v>
+        <v>60.27992789735976</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -537,7 +537,7 @@
         <v>0.3141880794689826</v>
       </c>
       <c r="H3" t="n">
-        <v>58.5</v>
+        <v>59.075</v>
       </c>
       <c r="I3" t="n">
         <v>30.24602026049204</v>
@@ -577,10 +577,10 @@
         <v>-4.499064189327432</v>
       </c>
       <c r="H4" t="n">
-        <v>58.87</v>
+        <v>57.5</v>
       </c>
       <c r="I4" t="n">
-        <v>29.64104822726272</v>
+        <v>24.84360089067966</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -617,7 +617,7 @@
         <v>-2.61443014217979</v>
       </c>
       <c r="H5" t="n">
-        <v>37.61</v>
+        <v>33.34</v>
       </c>
       <c r="I5" t="n">
         <v>0.7681175553823865</v>
@@ -658,10 +658,10 @@
         <v>1.221140364223394</v>
       </c>
       <c r="H6" t="n">
-        <v>48.9</v>
+        <v>49.83</v>
       </c>
       <c r="I6" t="n">
-        <v>7.685531821184766</v>
+        <v>3.700561976460603</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
         <v>1.286343944292292</v>
       </c>
       <c r="H7" t="n">
-        <v>52.23</v>
+        <v>48.4</v>
       </c>
       <c r="I7" t="n">
         <v>-0.7681175553823865</v>
@@ -738,7 +738,7 @@
         <v>-0.2571384120430241</v>
       </c>
       <c r="H8" t="n">
-        <v>55.62</v>
+        <v>50.985</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -779,10 +779,10 @@
         <v>0.0200984200212211</v>
       </c>
       <c r="H9" t="n">
-        <v>28.39</v>
+        <v>38.055</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1.402464938376533</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -820,7 +820,7 @@
         <v>0.167205430839917</v>
       </c>
       <c r="H10" t="n">
-        <v>49.2</v>
+        <v>44.905</v>
       </c>
       <c r="I10" t="n">
         <v>31.91298094210717</v>
@@ -856,11 +856,9 @@
       <c r="F11" t="n">
         <v>28.93</v>
       </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>35.59</v>
+        <v>31.8</v>
       </c>
       <c r="I11" t="n">
         <v>26.8173216074808</v>
@@ -900,7 +898,7 @@
         <v>-1.534037435719632</v>
       </c>
       <c r="H12" t="n">
-        <v>56.88</v>
+        <v>47.88</v>
       </c>
       <c r="I12" t="n">
         <v>11.39018691588785</v>
@@ -940,7 +938,7 @@
         <v>0.992020247858232</v>
       </c>
       <c r="H13" t="n">
-        <v>49.72</v>
+        <v>49.565</v>
       </c>
       <c r="I13" t="n">
         <v>-21.29982896987239</v>
@@ -980,7 +978,7 @@
         <v>-4.180016339930263</v>
       </c>
       <c r="H14" t="n">
-        <v>51.06</v>
+        <v>47.335</v>
       </c>
       <c r="I14" t="n">
         <v>-55.98714953271028</v>
@@ -1020,7 +1018,7 @@
         <v>0.06702962960133939</v>
       </c>
       <c r="H15" t="n">
-        <v>37.73</v>
+        <v>44.245</v>
       </c>
       <c r="I15" t="n">
         <v>10.19275700934578</v>
@@ -1060,7 +1058,7 @@
         <v>-3.231792280571145</v>
       </c>
       <c r="H16" t="n">
-        <v>46.9</v>
+        <v>50.87</v>
       </c>
       <c r="I16" t="n">
         <v>102.1028037383177</v>
@@ -1100,7 +1098,7 @@
         <v>-1.279081332956056</v>
       </c>
       <c r="H17" t="n">
-        <v>67.23999999999999</v>
+        <v>51.62</v>
       </c>
       <c r="I17" t="n">
         <v>-50.67172897196262</v>
@@ -1140,10 +1138,10 @@
         <v>-0.09337302073000636</v>
       </c>
       <c r="H18" t="n">
-        <v>52.67</v>
+        <v>56.305</v>
       </c>
       <c r="I18" t="n">
-        <v>-60.60339132349702</v>
+        <v>-62.06128724419467</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1180,7 +1178,7 @@
         <v>7.345106122639473</v>
       </c>
       <c r="H19" t="n">
-        <v>63.78</v>
+        <v>65.33500000000001</v>
       </c>
       <c r="I19" t="n">
         <v>31.967721911856</v>
@@ -1221,10 +1219,10 @@
         <v>-0.4410671269170658</v>
       </c>
       <c r="H20" t="n">
-        <v>31.13</v>
+        <v>35.98</v>
       </c>
       <c r="I20" t="n">
-        <v>-34.37568817441092</v>
+        <v>-36.80415650514261</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1261,7 +1259,7 @@
         <v>0.05908701218425355</v>
       </c>
       <c r="H21" t="n">
-        <v>31.28</v>
+        <v>34.555</v>
       </c>
       <c r="I21" t="n">
         <v>53.7429285620313</v>
@@ -1301,7 +1299,7 @@
         <v>5.422883218663305</v>
       </c>
       <c r="H22" t="n">
-        <v>35.8</v>
+        <v>30.585</v>
       </c>
       <c r="I22" t="n">
         <v>51.73104753423134</v>
@@ -1341,7 +1339,7 @@
         <v>0.9391963078561093</v>
       </c>
       <c r="H23" t="n">
-        <v>33.6</v>
+        <v>36.77500000000001</v>
       </c>
       <c r="I23" t="n">
         <v>25.43670264965651</v>
@@ -1381,7 +1379,7 @@
         <v>2.678399409785198</v>
       </c>
       <c r="H24" t="n">
-        <v>36.74</v>
+        <v>34.745</v>
       </c>
       <c r="I24" t="n">
         <v>7.301401869158878</v>
@@ -1421,7 +1419,7 @@
         <v>-3.965092371280805</v>
       </c>
       <c r="H25" t="n">
-        <v>33.3</v>
+        <v>28.41</v>
       </c>
       <c r="I25" t="n">
         <v>-50.96378504672898</v>
@@ -1462,10 +1460,10 @@
         <v>0.2619353681300373</v>
       </c>
       <c r="H26" t="n">
-        <v>41.07</v>
+        <v>50.41</v>
       </c>
       <c r="I26" t="n">
-        <v>25.20955574182733</v>
+        <v>26.96557586060348</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1502,7 +1500,7 @@
         <v>2.999175111211977</v>
       </c>
       <c r="H27" t="n">
-        <v>32.17</v>
+        <v>33.22</v>
       </c>
       <c r="I27" t="n">
         <v>-38.38547285149226</v>
@@ -1542,7 +1540,7 @@
         <v>1.843535171537232</v>
       </c>
       <c r="H28" t="n">
-        <v>50.95</v>
+        <v>41.055</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1582,10 +1580,10 @@
         <v>0.0614230582049048</v>
       </c>
       <c r="H29" t="n">
-        <v>30.35</v>
+        <v>43.625</v>
       </c>
       <c r="I29" t="n">
-        <v>46.5842414082146</v>
+        <v>48.64003399915002</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -1622,7 +1620,7 @@
         <v>0.07309772065891328</v>
       </c>
       <c r="H30" t="n">
-        <v>46.26</v>
+        <v>42.20999999999999</v>
       </c>
       <c r="I30" t="n">
         <v>-5.793707361775798</v>
@@ -1662,7 +1660,7 @@
         <v>0.00910553222430331</v>
       </c>
       <c r="H31" t="n">
-        <v>37.82</v>
+        <v>45.655</v>
       </c>
       <c r="I31" t="n">
         <v>90.84331009077752</v>
@@ -1702,10 +1700,10 @@
         <v>0.02084525007272494</v>
       </c>
       <c r="H32" t="n">
-        <v>13.03</v>
+        <v>12.38</v>
       </c>
       <c r="I32" t="n">
-        <v>-75.41911148365465</v>
+        <v>-75.07437314067148</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -1742,7 +1740,7 @@
         <v>0.4001945575069012</v>
       </c>
       <c r="H33" t="n">
-        <v>18.91</v>
+        <v>21.865</v>
       </c>
       <c r="I33" t="n">
         <v>-58.90014471780029</v>
@@ -1782,7 +1780,7 @@
         <v>0.2846199035338283</v>
       </c>
       <c r="H34" t="n">
-        <v>30.66</v>
+        <v>28.26</v>
       </c>
       <c r="I34" t="n">
         <v>-42.46910831570745</v>
@@ -1822,7 +1820,7 @@
         <v>-0.1028018435345398</v>
       </c>
       <c r="H35" t="n">
-        <v>40.79</v>
+        <v>37.19</v>
       </c>
       <c r="I35" t="n">
         <v>-34.07262021589793</v>
@@ -1862,10 +1860,10 @@
         <v>-7.063967310949983</v>
       </c>
       <c r="H36" t="n">
-        <v>38.27</v>
+        <v>47.49</v>
       </c>
       <c r="I36" t="n">
-        <v>74.74124642149307</v>
+        <v>68.27483829922593</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -1902,10 +1900,10 @@
         <v>0.06861811283803056</v>
       </c>
       <c r="H37" t="n">
-        <v>51.22</v>
+        <v>53.635</v>
       </c>
       <c r="I37" t="n">
-        <v>58.31314688394627</v>
+        <v>52.45467076662072</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -1942,10 +1940,10 @@
         <v>0.01328569587780193</v>
       </c>
       <c r="H38" t="n">
-        <v>45.41</v>
+        <v>55.345</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>-3.700561976460618</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -1982,7 +1980,7 @@
         <v>3.839131751270119</v>
       </c>
       <c r="H39" t="n">
-        <v>63.63</v>
+        <v>62.05</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -2022,7 +2020,7 @@
         <v>4.412519521183551</v>
       </c>
       <c r="H40" t="n">
-        <v>30.19</v>
+        <v>31.84</v>
       </c>
       <c r="I40" t="n">
         <v>44.33411214953271</v>
@@ -2062,7 +2060,7 @@
         <v>-6.151706657367163</v>
       </c>
       <c r="H41" t="n">
-        <v>50.59</v>
+        <v>52.28</v>
       </c>
       <c r="I41" t="n">
         <v>47.75116822429906</v>
@@ -2103,7 +2101,7 @@
         <v>0.1942386275072222</v>
       </c>
       <c r="H42" t="n">
-        <v>56.18</v>
+        <v>60.27500000000001</v>
       </c>
       <c r="I42" t="n">
         <v>41.71819497434547</v>
@@ -2143,7 +2141,7 @@
         <v>1.355289512628809</v>
       </c>
       <c r="H43" t="n">
-        <v>56.45</v>
+        <v>51.02</v>
       </c>
       <c r="I43" t="n">
         <v>1.492268967997133</v>
@@ -2184,7 +2182,7 @@
         <v>1.848273624075064</v>
       </c>
       <c r="H44" t="n">
-        <v>22.92</v>
+        <v>21.805</v>
       </c>
       <c r="I44" t="n">
         <v>-32.26692836113838</v>
@@ -2224,7 +2222,7 @@
         <v>0.9510909711578005</v>
       </c>
       <c r="H45" t="n">
-        <v>25.76</v>
+        <v>50.57</v>
       </c>
       <c r="I45" t="n">
         <v>-24.76635514018692</v>
@@ -2264,7 +2262,7 @@
         <v>0.03821387979852416</v>
       </c>
       <c r="H46" t="n">
-        <v>49</v>
+        <v>52.4</v>
       </c>
       <c r="I46" t="n">
         <v>43.10747663551401</v>
@@ -2304,7 +2302,7 @@
         <v>0.006574879059013327</v>
       </c>
       <c r="H47" t="n">
-        <v>36.03</v>
+        <v>44.31</v>
       </c>
       <c r="I47" t="n">
         <v>-39.16471962616824</v>
@@ -2344,7 +2342,7 @@
         <v>0.9056027172386589</v>
       </c>
       <c r="H48" t="n">
-        <v>51.42</v>
+        <v>53.7</v>
       </c>
       <c r="I48" t="n">
         <v>100.5788712011577</v>
@@ -2384,7 +2382,7 @@
         <v>-0.9664534641259643</v>
       </c>
       <c r="H49" t="n">
-        <v>51.73</v>
+        <v>56</v>
       </c>
       <c r="I49" t="n">
         <v>-73.74415887850468</v>
@@ -2424,7 +2422,7 @@
         <v>1.808627454139422</v>
       </c>
       <c r="H50" t="n">
-        <v>35.99</v>
+        <v>34.31</v>
       </c>
       <c r="I50" t="n">
         <v>-43.43862957724344</v>
@@ -2465,7 +2463,7 @@
         <v>2.794810104975634</v>
       </c>
       <c r="H51" t="n">
-        <v>50.51</v>
+        <v>49.11</v>
       </c>
       <c r="I51" t="n">
         <v>-36.30190359568073</v>
@@ -2505,7 +2503,7 @@
         <v>0.05299874823631171</v>
       </c>
       <c r="H52" t="n">
-        <v>36.42</v>
+        <v>45.585</v>
       </c>
       <c r="I52" t="n">
         <v>59.03170635442703</v>
@@ -2545,7 +2543,7 @@
         <v>0.3019460457018293</v>
       </c>
       <c r="H53" t="n">
-        <v>37.81</v>
+        <v>36.52</v>
       </c>
       <c r="I53" t="n">
         <v>-71.34929906542055</v>
@@ -2586,7 +2584,7 @@
         <v>5.641008076014133</v>
       </c>
       <c r="H54" t="n">
-        <v>55.53</v>
+        <v>62.555</v>
       </c>
       <c r="I54" t="n">
         <v>-6.084396467124634</v>
@@ -2626,7 +2624,7 @@
         <v>-0.5890244225007633</v>
       </c>
       <c r="H55" t="n">
-        <v>47.36</v>
+        <v>43.26</v>
       </c>
       <c r="I55" t="n">
         <v>39.59007551240561</v>
@@ -2666,7 +2664,7 @@
         <v>0.05443098966974722</v>
       </c>
       <c r="H56" t="n">
-        <v>65.98</v>
+        <v>50.11</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
@@ -2706,7 +2704,7 @@
         <v>-1.77053361249378</v>
       </c>
       <c r="H57" t="n">
-        <v>36.57</v>
+        <v>37.545</v>
       </c>
       <c r="I57" t="n">
         <v>-44.80685739730602</v>
@@ -2746,7 +2744,7 @@
         <v>-0.09143985264473488</v>
       </c>
       <c r="H58" t="n">
-        <v>36.76</v>
+        <v>35.885</v>
       </c>
       <c r="I58" t="n">
         <v>24.54153182308522</v>
@@ -2787,7 +2785,7 @@
         <v>1.572670875827523</v>
       </c>
       <c r="H59" t="n">
-        <v>43.71</v>
+        <v>46.535</v>
       </c>
       <c r="I59" t="n">
         <v>-3.913551401869168</v>
@@ -2827,7 +2825,7 @@
         <v>0.4646382763782856</v>
       </c>
       <c r="H60" t="n">
-        <v>30.67</v>
+        <v>34.485</v>
       </c>
       <c r="I60" t="n">
         <v>-10.42640186915888</v>
@@ -2867,7 +2865,7 @@
         <v>-0.03595279056427525</v>
       </c>
       <c r="H61" t="n">
-        <v>51.95</v>
+        <v>52.13</v>
       </c>
       <c r="I61" t="n">
         <v>5.793707361775784</v>
@@ -2907,10 +2905,10 @@
         <v>1.817983767525715</v>
       </c>
       <c r="H62" t="n">
-        <v>18.77</v>
+        <v>24.09</v>
       </c>
       <c r="I62" t="n">
-        <v>-32.17353005945826</v>
+        <v>-34.68349061605344</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
@@ -2947,7 +2945,7 @@
         <v>0.1300622866212008</v>
       </c>
       <c r="H63" t="n">
-        <v>61.37</v>
+        <v>60.765</v>
       </c>
       <c r="I63" t="n">
         <v>1.398711299701388</v>
@@ -2988,7 +2986,7 @@
         <v>-0.2694648852484086</v>
       </c>
       <c r="H64" t="n">
-        <v>34.84</v>
+        <v>43.58</v>
       </c>
       <c r="I64" t="n">
         <v>-62.58387054334956</v>
@@ -3028,7 +3026,7 @@
         <v>0.3282212496887102</v>
       </c>
       <c r="H65" t="n">
-        <v>20.78</v>
+        <v>28.565</v>
       </c>
       <c r="I65" t="n">
         <v>-45.3229838179187</v>
@@ -3068,7 +3066,7 @@
         <v>0.6329063689949501</v>
       </c>
       <c r="H66" t="n">
-        <v>30.92</v>
+        <v>31.5</v>
       </c>
       <c r="I66" t="n">
         <v>-74.89803973161426</v>
@@ -3108,7 +3106,7 @@
         <v>-0.02660402589146366</v>
       </c>
       <c r="H67" t="n">
-        <v>36.89</v>
+        <v>34.88500000000001</v>
       </c>
       <c r="I67" t="n">
         <v>-31.96772191185599</v>
@@ -3148,7 +3146,7 @@
         <v>0.175112852872738</v>
       </c>
       <c r="H68" t="n">
-        <v>46.21</v>
+        <v>50.585</v>
       </c>
       <c r="I68" t="n">
         <v>7.870461236506375</v>
@@ -3189,7 +3187,7 @@
         <v>0.05573417784977254</v>
       </c>
       <c r="H69" t="n">
-        <v>59.63</v>
+        <v>59.83</v>
       </c>
       <c r="I69" t="n">
         <v>58.45485917844818</v>
@@ -3229,7 +3227,7 @@
         <v>0.9521678733206076</v>
       </c>
       <c r="H70" t="n">
-        <v>54.44</v>
+        <v>44.12</v>
       </c>
       <c r="I70" t="n">
         <v>-31.42602693977513</v>
@@ -3269,7 +3267,7 @@
         <v>10.78154540867274</v>
       </c>
       <c r="H71" t="n">
-        <v>43.8</v>
+        <v>44.31</v>
       </c>
       <c r="I71" t="n">
         <v>-59.59033730379606</v>
@@ -3309,7 +3307,7 @@
         <v>-5.031547988302576</v>
       </c>
       <c r="H72" t="n">
-        <v>35.6</v>
+        <v>35.95</v>
       </c>
       <c r="I72" t="n">
         <v>3.971962616822428</v>
@@ -3349,7 +3347,7 @@
         <v>0.588510137595519</v>
       </c>
       <c r="H73" t="n">
-        <v>38.11</v>
+        <v>37.11499999999999</v>
       </c>
       <c r="I73" t="n">
         <v>-35.05933117583604</v>
@@ -3389,7 +3387,7 @@
         <v>-1.612606778720886</v>
       </c>
       <c r="H74" t="n">
-        <v>20.42</v>
+        <v>20.58</v>
       </c>
       <c r="I74" t="n">
         <v>-43.6623831775701</v>
@@ -3429,7 +3427,7 @@
         <v>6.488733930345523</v>
       </c>
       <c r="H75" t="n">
-        <v>37.33</v>
+        <v>50.86</v>
       </c>
       <c r="I75" t="n">
         <v>43.35967939441167</v>
@@ -3469,7 +3467,7 @@
         <v>-20.40097504287343</v>
       </c>
       <c r="H76" t="n">
-        <v>31.49</v>
+        <v>43.34</v>
       </c>
       <c r="I76" t="n">
         <v>-8.031542056074777</v>
@@ -3510,7 +3508,7 @@
         <v>10.45314512446346</v>
       </c>
       <c r="H77" t="n">
-        <v>58.34</v>
+        <v>50.5</v>
       </c>
       <c r="I77" t="n">
         <v>29.88979182901036</v>
@@ -3550,7 +3548,7 @@
         <v>-0.2368813254240325</v>
       </c>
       <c r="H78" t="n">
-        <v>60.68</v>
+        <v>54.025</v>
       </c>
       <c r="I78" t="n">
         <v>104.3808411214953</v>
@@ -3590,7 +3588,7 @@
         <v>0.7563625783740417</v>
       </c>
       <c r="H79" t="n">
-        <v>54.93</v>
+        <v>50.985</v>
       </c>
       <c r="I79" t="n">
         <v>60.42640186915887</v>
@@ -3630,7 +3628,7 @@
         <v>0.06115348347250073</v>
       </c>
       <c r="H80" t="n">
-        <v>32.7</v>
+        <v>33.97</v>
       </c>
       <c r="I80" t="n">
         <v>-53.48795397339087</v>
@@ -3671,7 +3669,7 @@
         <v>-3.608906905151208</v>
       </c>
       <c r="H81" t="n">
-        <v>37.85</v>
+        <v>47.26000000000001</v>
       </c>
       <c r="I81" t="n">
         <v>100.1460280373832</v>
@@ -3707,12 +3705,14 @@
       <c r="F82" t="n">
         <v>30.88</v>
       </c>
-      <c r="G82" t="inlineStr"/>
+      <c r="G82" t="n">
+        <v>0.09804152402695152</v>
+      </c>
       <c r="H82" t="n">
-        <v>41.13</v>
+        <v>37.225</v>
       </c>
       <c r="I82" t="n">
-        <v>-26.62409160977758</v>
+        <v>-29.33941257554872</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -3749,10 +3749,10 @@
         <v>0.8489189373413096</v>
       </c>
       <c r="H83" t="n">
-        <v>24.58</v>
+        <v>31.24</v>
       </c>
       <c r="I83" t="n">
-        <v>-20.57837384744342</v>
+        <v>-19.46451338716533</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
@@ -3789,7 +3789,7 @@
         <v>0.007417056977403794</v>
       </c>
       <c r="H84" t="n">
-        <v>54.79</v>
+        <v>37.655</v>
       </c>
       <c r="I84" t="n">
         <v>7.536800785083407</v>
@@ -3829,7 +3829,7 @@
         <v>3.000651602734764</v>
       </c>
       <c r="H85" t="n">
-        <v>34.17</v>
+        <v>31.715</v>
       </c>
       <c r="I85" t="n">
         <v>76.47677937113535</v>
@@ -3870,7 +3870,7 @@
         <v>0.2166615750083587</v>
       </c>
       <c r="H86" t="n">
-        <v>24.7</v>
+        <v>23.51</v>
       </c>
       <c r="I86" t="n">
         <v>-67.71679839697205</v>
@@ -3911,7 +3911,7 @@
         <v>1.638533052351645</v>
       </c>
       <c r="H87" t="n">
-        <v>48.97</v>
+        <v>50.555</v>
       </c>
       <c r="I87" t="n">
         <v>-11.95613088816972</v>
@@ -3951,7 +3951,7 @@
         <v>10.93458277277939</v>
       </c>
       <c r="H88" t="n">
-        <v>57.2</v>
+        <v>52.365</v>
       </c>
       <c r="I88" t="n">
         <v>23.66808109382366</v>
@@ -3991,7 +3991,7 @@
         <v>0.1674227036387368</v>
       </c>
       <c r="H89" t="n">
-        <v>51.58</v>
+        <v>49.445</v>
       </c>
       <c r="I89" t="n">
         <v>-9.790979097909796</v>
@@ -4032,7 +4032,7 @@
         <v>0.0839572651499547</v>
       </c>
       <c r="H90" t="n">
-        <v>26.55</v>
+        <v>27.58</v>
       </c>
       <c r="I90" t="n">
         <v>-73.34561241941849</v>
@@ -4072,10 +4072,10 @@
         <v>0.1660811237632738</v>
       </c>
       <c r="H91" t="n">
-        <v>46.4</v>
+        <v>48.83</v>
       </c>
       <c r="I91" t="n">
-        <v>-2.766135792120705</v>
+        <v>-1.402464938376548</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -4112,7 +4112,7 @@
         <v>0.1472024429514394</v>
       </c>
       <c r="H92" t="n">
-        <v>65.94</v>
+        <v>67.02</v>
       </c>
       <c r="I92" t="n">
         <v>-77.23983686357059</v>
@@ -4152,7 +4152,7 @@
         <v>-0.8454886074536311</v>
       </c>
       <c r="H93" t="n">
-        <v>46.1</v>
+        <v>35.19</v>
       </c>
       <c r="I93" t="n">
         <v>21.29982896987238</v>

</xml_diff>